<commit_message>
Comisión del almacén de 0,95 € por pedido confirmado en todo el modelo
Dashboard, Excel de contabilidad (parámetro, columna en Diario y línea en la
cuenta de resultados) y break-even del Excel de creativos (11,76 → 10,81 €).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/creativos/CeraLux_Creativos.xlsx
+++ b/creativos/CeraLux_Creativos.xlsx
@@ -1871,7 +1871,7 @@
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>14.34</c:v>
+                  <c:v>12.3495238095238</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-3.37</c:v>
@@ -1886,16 +1886,16 @@
                   <c:v>-2.84</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>37.66</c:v>
+                  <c:v>27.7076190476191</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>36.22</c:v>
+                  <c:v>30.2485714285714</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>-1.81</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16.19</c:v>
+                  <c:v>14.1995238095238</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>-0.05</c:v>
@@ -1904,7 +1904,7 @@
                   <c:v>-0.73</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-0.58</c:v>
+                  <c:v>-1.5752380952381</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1912,11 +1912,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="23218860"/>
-        <c:axId val="24872227"/>
+        <c:axId val="67037885"/>
+        <c:axId val="33948007"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="23218860"/>
+        <c:axId val="67037885"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1948,7 +1948,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24872227"/>
+        <c:crossAx val="33948007"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1956,7 +1956,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24872227"/>
+        <c:axId val="33948007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1998,7 +1998,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23218860"/>
+        <c:crossAx val="67037885"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,F3-C3+1)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>5</v>
@@ -2363,7 +2363,7 @@
       <c r="K7" s="8"/>
       <c r="L7" s="8" t="n">
         <f aca="false">F7*BEN_PEDIDO-B7*(1+RECARGO)</f>
-        <v>83.51</v>
+        <v>62.61</v>
       </c>
       <c r="M7" s="8"/>
     </row>
@@ -2397,7 +2397,7 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="n">
         <f aca="false">CPA_BE</f>
-        <v>11.76</v>
+        <v>10.81</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="11" t="n">
@@ -2472,12 +2472,12 @@
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="17" t="n">
         <f aca="false">COUNTIF(Creativos!$AA$5:$AA$16,"ESCALAR")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17" t="n">
         <f aca="false">COUNTIF(Creativos!$AA$5:$AA$16,"MANTENER")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="17"/>
       <c r="F14" s="17" t="n">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C18" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$B$5:$B$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>BROAD_H1 BOLARDO</v>
+        <v>BROAD_H2 LLAVES</v>
       </c>
       <c r="D18" s="20"/>
       <c r="E18" s="21" t="str">
@@ -2564,21 +2564,21 @@
       <c r="F18" s="21"/>
       <c r="G18" s="21" t="str">
         <f aca="false">IFERROR(IF(INDEX(Creativos!$I$5:$I$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0))="","[visual] "&amp;INDEX(Creativos!$H$5:$H$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),INDEX(Creativos!$I$5:$I$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0))),"")</f>
-        <v>[visual] Bolardo</v>
+        <v>[visual] Llaves</v>
       </c>
       <c r="H18" s="21"/>
       <c r="I18" s="21"/>
       <c r="J18" s="22" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$M$5:$M$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>85.54</v>
+        <v>37.7</v>
       </c>
       <c r="K18" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$S$5:$S$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>8.16518181818182</v>
+        <v>5.99772727272727</v>
       </c>
       <c r="L18" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>37.66</v>
+        <v>30.2485714285714</v>
       </c>
       <c r="M18" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C19" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$B$5:$B$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>BROAD_H2 LLAVES</v>
+        <v>BROAD_H1 BOLARDO</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="21" t="str">
@@ -2601,25 +2601,25 @@
       <c r="F19" s="21"/>
       <c r="G19" s="21" t="str">
         <f aca="false">IFERROR(IF(INDEX(Creativos!$I$5:$I$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0))="","[visual] "&amp;INDEX(Creativos!$H$5:$H$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),INDEX(Creativos!$I$5:$I$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0))),"")</f>
-        <v>[visual] Llaves</v>
+        <v>[visual] Bolardo</v>
       </c>
       <c r="H19" s="21"/>
       <c r="I19" s="21"/>
       <c r="J19" s="22" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$M$5:$M$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>37.7</v>
+        <v>85.54</v>
       </c>
       <c r="K19" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$S$5:$S$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>5.99772727272727</v>
+        <v>8.16518181818182</v>
       </c>
       <c r="L19" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>36.22</v>
+        <v>27.7076190476191</v>
       </c>
       <c r="M19" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>ESCALAR</v>
+        <v>MANTENER</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="L20" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,3),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>16.19</v>
+        <v>14.1995238095238</v>
       </c>
       <c r="M20" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,3),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="L21" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,4),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>14.34</v>
+        <v>12.3495238095238</v>
       </c>
       <c r="M21" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,4),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="K26" s="23" t="n">
         <f aca="false">I26*BEN_PEDIDO-G26*(1+RECARGO)</f>
-        <v>10.97</v>
+        <v>8.97952380952381</v>
       </c>
       <c r="L26" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$D$5:$D$5000,$B26,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$D$5:$D$5000,$B26,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="K28" s="23" t="n">
         <f aca="false">I28*BEN_PEDIDO-G28*(1+RECARGO)</f>
-        <v>86.9</v>
+        <v>67.9904761904762</v>
       </c>
       <c r="L28" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$D$5:$D$5000,$B28,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$D$5:$D$5000,$B28,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="K32" s="23" t="n">
         <f aca="false">I32*BEN_PEDIDO-G32*(1+RECARGO)</f>
-        <v>10.97</v>
+        <v>8.97952380952381</v>
       </c>
       <c r="L32" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$R$5:$R$5000,LEFT($B32,FIND(" · ",$B32&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B32,FIND(" · ",$B32&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="K34" s="23" t="n">
         <f aca="false">I34*BEN_PEDIDO-G34*(1+RECARGO)</f>
-        <v>86.9</v>
+        <v>67.9904761904762</v>
       </c>
       <c r="L34" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$R$5:$R$5000,LEFT($B34,FIND(" · ",$B34&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B34,FIND(" · ",$B34&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="K38" s="23" t="n">
         <f aca="false">I38*BEN_PEDIDO-G38*(1+RECARGO)</f>
-        <v>10.97</v>
+        <v>8.97952380952381</v>
       </c>
       <c r="L38" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="K40" s="23" t="n">
         <f aca="false">I40*BEN_PEDIDO-G40*(1+RECARGO)</f>
-        <v>37.66</v>
+        <v>27.7076190476191</v>
       </c>
       <c r="L40" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="K41" s="23" t="n">
         <f aca="false">I41*BEN_PEDIDO-G41*(1+RECARGO)</f>
-        <v>34.41</v>
+        <v>28.4385714285714</v>
       </c>
       <c r="L41" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="K42" s="23" t="n">
         <f aca="false">I42*BEN_PEDIDO-G42*(1+RECARGO)</f>
-        <v>16.14</v>
+        <v>14.1495238095238</v>
       </c>
       <c r="L42" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="K43" s="23" t="n">
         <f aca="false">I43*BEN_PEDIDO-G43*(1+RECARGO)</f>
-        <v>-1.31</v>
+        <v>-2.3052380952381</v>
       </c>
       <c r="L43" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="H6" s="23" t="n">
         <f aca="false">Creativos!T5</f>
-        <v>14.34</v>
+        <v>12.3495238095238</v>
       </c>
       <c r="I6" s="24" t="str">
         <f aca="false">Creativos!AA5</f>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H8" s="33" t="n">
         <f aca="false">SUM(H6:H7)</f>
-        <v>10.97</v>
+        <v>8.97952380952381</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3921,11 +3921,11 @@
       </c>
       <c r="H19" s="23" t="n">
         <f aca="false">Creativos!T10</f>
-        <v>37.66</v>
+        <v>27.7076190476191</v>
       </c>
       <c r="I19" s="24" t="str">
         <f aca="false">Creativos!AA10</f>
-        <v>ESCALAR</v>
+        <v>MANTENER</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">Creativos!T11</f>
-        <v>36.22</v>
+        <v>30.2485714285714</v>
       </c>
       <c r="I20" s="24" t="str">
         <f aca="false">Creativos!AA11</f>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">Creativos!T13</f>
-        <v>16.19</v>
+        <v>14.1995238095238</v>
       </c>
       <c r="I22" s="24" t="str">
         <f aca="false">Creativos!AA13</f>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="H25" s="23" t="n">
         <f aca="false">Creativos!T16</f>
-        <v>-0.58</v>
+        <v>-1.5752380952381</v>
       </c>
       <c r="I25" s="24" t="str">
         <f aca="false">Creativos!AA16</f>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="H26" s="33" t="n">
         <f aca="false">SUM(H19:H25)</f>
-        <v>86.9</v>
+        <v>67.9904761904762</v>
       </c>
     </row>
   </sheetData>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="T5" s="23" t="n">
         <f aca="false">R5*BEN_PEDIDO-M5*(1+RECARGO)</f>
-        <v>14.34</v>
+        <v>12.3495238095238</v>
       </c>
       <c r="U5" s="27" t="n">
         <f aca="false">IF(N5&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A5,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N5,"")</f>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="AC5" s="47" t="n">
         <f aca="false">IF(M5&gt;0,T5+ROW()/1000000,-1000000+ROW())</f>
-        <v>14.340005</v>
+        <v>12.3495288095238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="T10" s="23" t="n">
         <f aca="false">R10*BEN_PEDIDO-M10*(1+RECARGO)</f>
-        <v>37.66</v>
+        <v>27.7076190476191</v>
       </c>
       <c r="U10" s="27" t="n">
         <f aca="false">IF(N10&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A10,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N10,"")</f>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="AA10" s="19" t="str">
         <f aca="false">IF(M10=0,"SIN GASTO",IF(Q10=0,IF(M10&gt;=APG_SV*CPA_BE,"APAGAR",IF(M10&gt;=0.5*CPA_BE,"VIGILAR","APRENDIENDO")),IF(AND(S10&lt;=UMB_ESC*CPA_BE,Q10&gt;=3),"ESCALAR",IF(AND(S10&lt;=CPA_BE,Q10&gt;=3),"MANTENER",IF(S10&lt;=CPA_BE,"PROMETEDOR",IF(M10&gt;=APG_CV*CPA_BE,"APAGAR","VIGILAR"))))))</f>
-        <v>ESCALAR</v>
+        <v>MANTENER</v>
       </c>
       <c r="AB10" s="31" t="str">
         <f aca="false">IF(N10&lt;MIN_IMPR,"Pocos datos todavía",IF(AND(ISNUMBER(U10),U10&lt;0.7*MEDIA_GANCHO),"Gancho flojo: cambia los 3 primeros segundos",IF(AND(ISNUMBER(W10),W10&lt;0.7*MEDIA_CTR),"Enganchan pero no hacen clic: refuerza oferta y llamada a la acción",IF(AND(O10&gt;=20,ISNUMBER(Y10),Y10&lt;0.6*MEDIA_CVR),"Hacen clic pero no compran: revisa ángulo y página",IF(AND(ISNUMBER(U10),U10&gt;=1.3*MEDIA_GANCHO),"Gancho por encima de la media: reutiliza este inicio","En la media de la campaña")))))</f>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="AC10" s="47" t="n">
         <f aca="false">IF(M10&gt;0,T10+ROW()/1000000,-1000000+ROW())</f>
-        <v>37.66001</v>
+        <v>27.7076290476191</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="T11" s="23" t="n">
         <f aca="false">R11*BEN_PEDIDO-M11*(1+RECARGO)</f>
-        <v>36.22</v>
+        <v>30.2485714285714</v>
       </c>
       <c r="U11" s="27" t="n">
         <f aca="false">IF(N11&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A11,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N11,"")</f>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="AC11" s="47" t="n">
         <f aca="false">IF(M11&gt;0,T11+ROW()/1000000,-1000000+ROW())</f>
-        <v>36.220011</v>
+        <v>30.2485824285714</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="T13" s="23" t="n">
         <f aca="false">R13*BEN_PEDIDO-M13*(1+RECARGO)</f>
-        <v>16.19</v>
+        <v>14.1995238095238</v>
       </c>
       <c r="U13" s="27" t="n">
         <f aca="false">IF(N13&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A13,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N13,"")</f>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="AC13" s="47" t="n">
         <f aca="false">IF(M13&gt;0,T13+ROW()/1000000,-1000000+ROW())</f>
-        <v>16.190013</v>
+        <v>14.1995368095238</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="T16" s="23" t="n">
         <f aca="false">R16*BEN_PEDIDO-M16*(1+RECARGO)</f>
-        <v>-0.58</v>
+        <v>-1.5752380952381</v>
       </c>
       <c r="U16" s="27" t="n">
         <f aca="false">IF(N16&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A16,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N16,"")</f>
@@ -5602,7 +5602,7 @@
       </c>
       <c r="AC16" s="47" t="n">
         <f aca="false">IF(M16&gt;0,T16+ROW()/1000000,-1000000+ROW())</f>
-        <v>-0.579984</v>
+        <v>-1.5752220952381</v>
       </c>
     </row>
   </sheetData>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="T5" s="23" t="n">
         <f aca="false">IF(A5="","",R5*RATIO*BEN_PEDIDO-Q5*(1+RECARGO))</f>
-        <v>10.97</v>
+        <v>8.97952380952381</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="T7" s="23" t="n">
         <f aca="false">IF(A7="","",R7*RATIO*BEN_PEDIDO-Q7*(1+RECARGO))</f>
-        <v>86.9</v>
+        <v>67.9904761904762</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9542,7 +9542,7 @@
         <v>194</v>
       </c>
       <c r="C4" s="63" t="n">
-        <v>11.76</v>
+        <v>10.81</v>
       </c>
       <c r="E4" s="64" t="s">
         <v>195</v>
@@ -9556,7 +9556,7 @@
         <v>197</v>
       </c>
       <c r="C5" s="63" t="n">
-        <v>11.76</v>
+        <v>10.81</v>
       </c>
       <c r="E5" s="64" t="s">
         <v>198</v>

</xml_diff>

<commit_message>
Tres packs: Pack 3 (3 uds, 49,99 €) en panel, importadores y Excel
El panel, los dos importadores y Shopify en directo clasifican por unidades
(1, 2, 3 o más). El Excel de contabilidad pasa a tener Pack 3 en Config y en el
Diario (columnas reordenadas). Mismos totales que antes con los datos sin Pack 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/creativos/CeraLux_Creativos.xlsx
+++ b/creativos/CeraLux_Creativos.xlsx
@@ -1871,7 +1871,7 @@
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>12.3495238095238</c:v>
+                  <c:v>13.2295238095238</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-3.37</c:v>
@@ -1886,16 +1886,16 @@
                   <c:v>-2.84</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27.7076190476191</c:v>
+                  <c:v>32.1076190476191</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30.2485714285714</c:v>
+                  <c:v>32.8885714285714</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>-1.81</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>14.1995238095238</c:v>
+                  <c:v>15.0795238095238</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>-0.05</c:v>
@@ -1904,7 +1904,7 @@
                   <c:v>-0.73</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1.5752380952381</c:v>
+                  <c:v>-1.13523809523809</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1912,11 +1912,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="67037885"/>
-        <c:axId val="33948007"/>
+        <c:axId val="7514643"/>
+        <c:axId val="10726682"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="67037885"/>
+        <c:axId val="7514643"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1948,7 +1948,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33948007"/>
+        <c:crossAx val="10726682"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1956,7 +1956,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33948007"/>
+        <c:axId val="10726682"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1998,7 +1998,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67037885"/>
+        <c:crossAx val="7514643"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2363,7 +2363,7 @@
       <c r="K7" s="8"/>
       <c r="L7" s="8" t="n">
         <f aca="false">F7*BEN_PEDIDO-B7*(1+RECARGO)</f>
-        <v>62.61</v>
+        <v>71.85</v>
       </c>
       <c r="M7" s="8"/>
     </row>
@@ -2397,7 +2397,7 @@
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="n">
         <f aca="false">CPA_BE</f>
-        <v>10.81</v>
+        <v>11.23</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="11" t="n">
@@ -2472,12 +2472,12 @@
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="17" t="n">
         <f aca="false">COUNTIF(Creativos!$AA$5:$AA$16,"ESCALAR")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17" t="n">
         <f aca="false">COUNTIF(Creativos!$AA$5:$AA$16,"MANTENER")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="17"/>
       <c r="F14" s="17" t="n">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="L18" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>30.2485714285714</v>
+        <v>32.8885714285714</v>
       </c>
       <c r="M18" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,1),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2615,11 +2615,11 @@
       </c>
       <c r="L19" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>27.7076190476191</v>
+        <v>32.1076190476191</v>
       </c>
       <c r="M19" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,2),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>MANTENER</v>
+        <v>ESCALAR</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="L20" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,3),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>14.1995238095238</v>
+        <v>15.0795238095238</v>
       </c>
       <c r="M20" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,3),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="L21" s="23" t="n">
         <f aca="false">IFERROR(INDEX(Creativos!$T$5:$T$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,4),Creativos!$AC$5:$AC$16,0)),"")</f>
-        <v>12.3495238095238</v>
+        <v>13.2295238095238</v>
       </c>
       <c r="M21" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Creativos!$AA$5:$AA$16,MATCH(LARGE(Creativos!$AC$5:$AC$16,4),Creativos!$AC$5:$AC$16,0)),"")</f>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="K26" s="23" t="n">
         <f aca="false">I26*BEN_PEDIDO-G26*(1+RECARGO)</f>
-        <v>8.97952380952381</v>
+        <v>9.85952380952381</v>
       </c>
       <c r="L26" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$D$5:$D$5000,$B26,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$D$5:$D$5000,$B26,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="K28" s="23" t="n">
         <f aca="false">I28*BEN_PEDIDO-G28*(1+RECARGO)</f>
-        <v>67.9904761904762</v>
+        <v>76.3504761904762</v>
       </c>
       <c r="L28" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$D$5:$D$5000,$B28,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$D$5:$D$5000,$B28,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="K32" s="23" t="n">
         <f aca="false">I32*BEN_PEDIDO-G32*(1+RECARGO)</f>
-        <v>8.97952380952381</v>
+        <v>9.85952380952381</v>
       </c>
       <c r="L32" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$R$5:$R$5000,LEFT($B32,FIND(" · ",$B32&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B32,FIND(" · ",$B32&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="K34" s="23" t="n">
         <f aca="false">I34*BEN_PEDIDO-G34*(1+RECARGO)</f>
-        <v>67.9904761904762</v>
+        <v>76.3504761904762</v>
       </c>
       <c r="L34" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$R$5:$R$5000,LEFT($B34,FIND(" · ",$B34&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B34,FIND(" · ",$B34&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="K38" s="23" t="n">
         <f aca="false">I38*BEN_PEDIDO-G38*(1+RECARGO)</f>
-        <v>8.97952380952381</v>
+        <v>9.85952380952381</v>
       </c>
       <c r="L38" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="K40" s="23" t="n">
         <f aca="false">I40*BEN_PEDIDO-G40*(1+RECARGO)</f>
-        <v>27.7076190476191</v>
+        <v>32.1076190476191</v>
       </c>
       <c r="L40" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="K41" s="23" t="n">
         <f aca="false">I41*BEN_PEDIDO-G41*(1+RECARGO)</f>
-        <v>28.4385714285714</v>
+        <v>31.0785714285714</v>
       </c>
       <c r="L41" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="K42" s="23" t="n">
         <f aca="false">I42*BEN_PEDIDO-G42*(1+RECARGO)</f>
-        <v>14.1495238095238</v>
+        <v>15.0295238095238</v>
       </c>
       <c r="L42" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="K43" s="23" t="n">
         <f aca="false">I43*BEN_PEDIDO-G43*(1+RECARGO)</f>
-        <v>-2.3052380952381</v>
+        <v>-1.86523809523809</v>
       </c>
       <c r="L43" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="H6" s="23" t="n">
         <f aca="false">Creativos!T5</f>
-        <v>12.3495238095238</v>
+        <v>13.2295238095238</v>
       </c>
       <c r="I6" s="24" t="str">
         <f aca="false">Creativos!AA5</f>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="H8" s="33" t="n">
         <f aca="false">SUM(H6:H7)</f>
-        <v>8.97952380952381</v>
+        <v>9.85952380952381</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3921,11 +3921,11 @@
       </c>
       <c r="H19" s="23" t="n">
         <f aca="false">Creativos!T10</f>
-        <v>27.7076190476191</v>
+        <v>32.1076190476191</v>
       </c>
       <c r="I19" s="24" t="str">
         <f aca="false">Creativos!AA10</f>
-        <v>MANTENER</v>
+        <v>ESCALAR</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">Creativos!T11</f>
-        <v>30.2485714285714</v>
+        <v>32.8885714285714</v>
       </c>
       <c r="I20" s="24" t="str">
         <f aca="false">Creativos!AA11</f>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">Creativos!T13</f>
-        <v>14.1995238095238</v>
+        <v>15.0795238095238</v>
       </c>
       <c r="I22" s="24" t="str">
         <f aca="false">Creativos!AA13</f>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="H25" s="23" t="n">
         <f aca="false">Creativos!T16</f>
-        <v>-1.5752380952381</v>
+        <v>-1.13523809523809</v>
       </c>
       <c r="I25" s="24" t="str">
         <f aca="false">Creativos!AA16</f>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="H26" s="33" t="n">
         <f aca="false">SUM(H19:H25)</f>
-        <v>67.9904761904762</v>
+        <v>76.3504761904762</v>
       </c>
     </row>
   </sheetData>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="T5" s="23" t="n">
         <f aca="false">R5*BEN_PEDIDO-M5*(1+RECARGO)</f>
-        <v>12.3495238095238</v>
+        <v>13.2295238095238</v>
       </c>
       <c r="U5" s="27" t="n">
         <f aca="false">IF(N5&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A5,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N5,"")</f>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="AC5" s="47" t="n">
         <f aca="false">IF(M5&gt;0,T5+ROW()/1000000,-1000000+ROW())</f>
-        <v>12.3495288095238</v>
+        <v>13.2295288095238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="T10" s="23" t="n">
         <f aca="false">R10*BEN_PEDIDO-M10*(1+RECARGO)</f>
-        <v>27.7076190476191</v>
+        <v>32.1076190476191</v>
       </c>
       <c r="U10" s="27" t="n">
         <f aca="false">IF(N10&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A10,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N10,"")</f>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="AA10" s="19" t="str">
         <f aca="false">IF(M10=0,"SIN GASTO",IF(Q10=0,IF(M10&gt;=APG_SV*CPA_BE,"APAGAR",IF(M10&gt;=0.5*CPA_BE,"VIGILAR","APRENDIENDO")),IF(AND(S10&lt;=UMB_ESC*CPA_BE,Q10&gt;=3),"ESCALAR",IF(AND(S10&lt;=CPA_BE,Q10&gt;=3),"MANTENER",IF(S10&lt;=CPA_BE,"PROMETEDOR",IF(M10&gt;=APG_CV*CPA_BE,"APAGAR","VIGILAR"))))))</f>
-        <v>MANTENER</v>
+        <v>ESCALAR</v>
       </c>
       <c r="AB10" s="31" t="str">
         <f aca="false">IF(N10&lt;MIN_IMPR,"Pocos datos todavía",IF(AND(ISNUMBER(U10),U10&lt;0.7*MEDIA_GANCHO),"Gancho flojo: cambia los 3 primeros segundos",IF(AND(ISNUMBER(W10),W10&lt;0.7*MEDIA_CTR),"Enganchan pero no hacen clic: refuerza oferta y llamada a la acción",IF(AND(O10&gt;=20,ISNUMBER(Y10),Y10&lt;0.6*MEDIA_CVR),"Hacen clic pero no compran: revisa ángulo y página",IF(AND(ISNUMBER(U10),U10&gt;=1.3*MEDIA_GANCHO),"Gancho por encima de la media: reutiliza este inicio","En la media de la campaña")))))</f>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="AC10" s="47" t="n">
         <f aca="false">IF(M10&gt;0,T10+ROW()/1000000,-1000000+ROW())</f>
-        <v>27.7076290476191</v>
+        <v>32.1076290476191</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="T11" s="23" t="n">
         <f aca="false">R11*BEN_PEDIDO-M11*(1+RECARGO)</f>
-        <v>30.2485714285714</v>
+        <v>32.8885714285714</v>
       </c>
       <c r="U11" s="27" t="n">
         <f aca="false">IF(N11&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A11,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N11,"")</f>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="AC11" s="47" t="n">
         <f aca="false">IF(M11&gt;0,T11+ROW()/1000000,-1000000+ROW())</f>
-        <v>30.2485824285714</v>
+        <v>32.8885824285714</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="T13" s="23" t="n">
         <f aca="false">R13*BEN_PEDIDO-M13*(1+RECARGO)</f>
-        <v>14.1995238095238</v>
+        <v>15.0795238095238</v>
       </c>
       <c r="U13" s="27" t="n">
         <f aca="false">IF(N13&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A13,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N13,"")</f>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="AC13" s="47" t="n">
         <f aca="false">IF(M13&gt;0,T13+ROW()/1000000,-1000000+ROW())</f>
-        <v>14.1995368095238</v>
+        <v>15.0795368095238</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="T16" s="23" t="n">
         <f aca="false">R16*BEN_PEDIDO-M16*(1+RECARGO)</f>
-        <v>-1.5752380952381</v>
+        <v>-1.13523809523809</v>
       </c>
       <c r="U16" s="27" t="n">
         <f aca="false">IF(N16&gt;0,SUMIFS(Histórico!$M$5:$M$5000,Histórico!$B$5:$B$5000,$A16,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/N16,"")</f>
@@ -5602,7 +5602,7 @@
       </c>
       <c r="AC16" s="47" t="n">
         <f aca="false">IF(M16&gt;0,T16+ROW()/1000000,-1000000+ROW())</f>
-        <v>-1.5752220952381</v>
+        <v>-1.13522209523809</v>
       </c>
     </row>
   </sheetData>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="T5" s="23" t="n">
         <f aca="false">IF(A5="","",R5*RATIO*BEN_PEDIDO-Q5*(1+RECARGO))</f>
-        <v>8.97952380952381</v>
+        <v>9.85952380952381</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="T7" s="23" t="n">
         <f aca="false">IF(A7="","",R7*RATIO*BEN_PEDIDO-Q7*(1+RECARGO))</f>
-        <v>67.9904761904762</v>
+        <v>76.3504761904762</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9542,7 +9542,7 @@
         <v>194</v>
       </c>
       <c r="C4" s="63" t="n">
-        <v>10.81</v>
+        <v>11.23</v>
       </c>
       <c r="E4" s="64" t="s">
         <v>195</v>
@@ -9556,7 +9556,7 @@
         <v>197</v>
       </c>
       <c r="C5" s="63" t="n">
-        <v>10.81</v>
+        <v>11.23</v>
       </c>
       <c r="E5" s="64" t="s">
         <v>198</v>

</xml_diff>

<commit_message>
Nomenclatura de anuncios ÁNGULO_CUERPO_VISUAL_HOOK_VN y cuerpo C4
- generar_creativos.py lee el nombre (p. ej. BROAD_C4_BOLARDO_PRECIO_V1) y
  rellena cuerpo, formato, concepto, tipo y hook vacíos; toma el último
  nombre de Meta si se renombra.
- biblioteca.json: cuerpo C4 (demo + uña + oferta octubre) y textos de los
  hooks PRECIO / MIRA / TIENES.
- Guion DEMO y guía del Excel con los nombres nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFjE4yx23BY3D6kaMQowKe
</commit_message>
<xml_diff>
--- a/creativos/CeraLux_Creativos.xlsx
+++ b/creativos/CeraLux_Creativos.xlsx
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="253">
   <si>
     <t xml:space="preserve">CeraLux · Creativos</t>
   </si>
@@ -243,6 +243,9 @@
     <t xml:space="preserve">C3 · Demostración real · sin cortes</t>
   </si>
   <si>
+    <t xml:space="preserve">C4 · Demo · uña + oferta octubre</t>
+  </si>
+  <si>
     <t xml:space="preserve">POR CONCEPTO DE HOOK</t>
   </si>
   <si>
@@ -597,6 +600,39 @@
     <t xml:space="preserve">El precio del Pack 2 en la tienda es 39,99 €.</t>
   </si>
   <si>
+    <t xml:space="preserve">C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo · uña + oferta octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BROAD — demostración + oferta de lanzamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demostración real (UGC) + voz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y eso sin quedarte tirado dos días sin coche. Y sí, ya lo has probado: la pasta de dientes, lo del súper, los rotuladores esos que anuncian... y la raya ahí sigue.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dos pulsaciones sobre el paño, y lo pasamos directamente por encima del arañazo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La fórmula de nanopolímeros rellena la marca y te alisa la superficie al instante, sin estropear el barniz. ¿Esa raya blanca que ves cada vez que te acercas al coche? Un par de pasadas, y deja de verse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te preguntarás si te va a servir a ti. Pasa la uña por la raya. Si no se engancha, esto es para ti. Si se engancha, es de taller. Así de claro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por su lanzamiento, solo hasta el 31 de octubre, te llevas dos botes por 39,90. El segundo te sale a menos de diez euros. Envío gratis, y no pagas nada hasta que te llega a casa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulsa el enlace de abajo y pídelo ahora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Va detrás de los hooks PRECIO, MIRA y TIENES sobre el visual BOLARDO (guion: creativos/guiones/guion_DEMO_3hooks.txt). Necesita el Pack 2 a 39,90 € en EasySell.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Matriz hook × cuerpo: CPA real de cada combinación</t>
   </si>
   <si>
@@ -807,7 +843,7 @@
     <t xml:space="preserve">Para sacarle partido</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombra los anuncios ÁNGULO_CONCEPTO_HOOK_VERSIÓN (ej.: BROAD_LLAVES_H2_V3). Así cada variación se agrupa sola por concepto.</t>
+    <t xml:space="preserve">Nombra los anuncios ÁNGULO_CUERPO_VISUAL_HOOK_VERSIÓN (ej.: BROAD_C4_BOLARDO_PRECIO_V1; MUDO si la voz no dice hook). Con ese nombre el cuerpo, el concepto y el hook se rellenan solos al regenerar. Mismo nombre en el vídeo del PC.</t>
   </si>
   <si>
     <t xml:space="preserve">Testea hooks nuevos sobre un cuerpo ganador (mismo cuerpo, distinto inicio): así sabes si lo que gana es el hook o el cuerpo.</t>
@@ -1912,11 +1948,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="7514643"/>
-        <c:axId val="10726682"/>
+        <c:axId val="79447543"/>
+        <c:axId val="37681830"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="7514643"/>
+        <c:axId val="79447543"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1948,7 +1984,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10726682"/>
+        <c:crossAx val="37681830"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1956,7 +1992,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10726682"/>
+        <c:axId val="37681830"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1998,7 +2034,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7514643"/>
+        <c:crossAx val="79447543"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2032,14 +2068,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>430200</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>7560</xdr:rowOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2047,7 +2083,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="141120" y="10172880"/>
+        <a:off x="141120" y="10372680"/>
         <a:ext cx="11159640" cy="2807640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2245,7 +2281,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:M84"/>
+  <dimension ref="B1:M85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2278,7 +2314,7 @@
       </c>
       <c r="F3" s="4" t="n">
         <f aca="true">TODAY()</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="3" t="s">
@@ -2286,7 +2322,7 @@
       </c>
       <c r="I3" s="5" t="n">
         <f aca="false">MAX(1,F3-C3+1)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>5</v>
@@ -3071,93 +3107,93 @@
         <v>0.0178562496873906</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6" t="s">
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-    </row>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="25" t="n">
+        <f aca="false">COUNTIF(Creativos!$E$5:$E$16,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1))</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="25" t="n">
+        <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="26" t="n">
+        <f aca="false">H35*RATIO</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="23" t="str">
+        <f aca="false">IF(I35&gt;0,G35/I35,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="23" t="n">
+        <f aca="false">I35*BEN_PEDIDO-G35*(1+RECARGO)</f>
+        <v>0</v>
+      </c>
+      <c r="L35" s="27" t="str">
+        <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="27" t="str">
+        <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$R$5:$R$5000,LEFT($B35,FIND(" · ",$B35&amp;" · ")-1),Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18" t="s">
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="G37" s="18" t="s">
+      <c r="G38" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="H37" s="18" t="s">
+      <c r="H38" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="I37" s="18" t="s">
+      <c r="I38" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J37" s="18" t="s">
+      <c r="J38" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="K37" s="18" t="s">
+      <c r="K38" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="L37" s="18" t="s">
+      <c r="L38" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="M37" s="18" t="s">
+      <c r="M38" s="18" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="25" t="n">
-        <f aca="false">COUNTIF(Creativos!$H$5:$H$16,$B38)</f>
-        <v>2</v>
-      </c>
-      <c r="G38" s="22" t="n">
-        <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>13.67</v>
-      </c>
-      <c r="H38" s="25" t="n">
-        <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>2</v>
-      </c>
-      <c r="I38" s="26" t="n">
-        <f aca="false">H38*RATIO</f>
-        <v>2.0952380952381</v>
-      </c>
-      <c r="J38" s="23" t="n">
-        <f aca="false">IF(I38&gt;0,G38/I38,"")</f>
-        <v>6.52431818181818</v>
-      </c>
-      <c r="K38" s="23" t="n">
-        <f aca="false">I38*BEN_PEDIDO-G38*(1+RECARGO)</f>
-        <v>9.85952380952381</v>
-      </c>
-      <c r="L38" s="27" t="n">
-        <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.253694581280788</v>
-      </c>
-      <c r="M38" s="27" t="n">
-        <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B38,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.0254515599343186</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3169,35 +3205,35 @@
       <c r="E39" s="20"/>
       <c r="F39" s="25" t="n">
         <f aca="false">COUNTIF(Creativos!$H$5:$H$16,$B39)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" s="22" t="n">
         <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>14.36</v>
+        <v>13.67</v>
       </c>
       <c r="H39" s="25" t="n">
         <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I39" s="26" t="n">
         <f aca="false">H39*RATIO</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="23" t="str">
+        <v>2.0952380952381</v>
+      </c>
+      <c r="J39" s="23" t="n">
         <f aca="false">IF(I39&gt;0,G39/I39,"")</f>
-        <v/>
+        <v>6.52431818181818</v>
       </c>
       <c r="K39" s="23" t="n">
         <f aca="false">I39*BEN_PEDIDO-G39*(1+RECARGO)</f>
-        <v>-14.36</v>
+        <v>9.85952380952381</v>
       </c>
       <c r="L39" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.192771084337349</v>
+        <v>0.253694581280788</v>
       </c>
       <c r="M39" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B39,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.0315106580166821</v>
+        <v>0.0254515599343186</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3209,35 +3245,35 @@
       <c r="E40" s="20"/>
       <c r="F40" s="25" t="n">
         <f aca="false">COUNTIF(Creativos!$H$5:$H$16,$B40)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G40" s="22" t="n">
         <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>85.54</v>
+        <v>14.36</v>
       </c>
       <c r="H40" s="25" t="n">
         <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I40" s="26" t="n">
         <f aca="false">H40*RATIO</f>
-        <v>10.4761904761905</v>
-      </c>
-      <c r="J40" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="23" t="str">
         <f aca="false">IF(I40&gt;0,G40/I40,"")</f>
-        <v>8.16518181818182</v>
+        <v/>
       </c>
       <c r="K40" s="23" t="n">
         <f aca="false">I40*BEN_PEDIDO-G40*(1+RECARGO)</f>
-        <v>32.1076190476191</v>
+        <v>-14.36</v>
       </c>
       <c r="L40" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.121081615362892</v>
+        <v>0.192771084337349</v>
       </c>
       <c r="M40" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B40,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.0160971476983903</v>
+        <v>0.0315106580166821</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3249,35 +3285,35 @@
       <c r="E41" s="20"/>
       <c r="F41" s="25" t="n">
         <f aca="false">COUNTIF(Creativos!$H$5:$H$16,$B41)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="22" t="n">
         <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>39.51</v>
+        <v>85.54</v>
       </c>
       <c r="H41" s="25" t="n">
         <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I41" s="26" t="n">
         <f aca="false">H41*RATIO</f>
-        <v>6.28571428571429</v>
+        <v>10.4761904761905</v>
       </c>
       <c r="J41" s="23" t="n">
         <f aca="false">IF(I41&gt;0,G41/I41,"")</f>
-        <v>6.28568181818182</v>
+        <v>8.16518181818182</v>
       </c>
       <c r="K41" s="23" t="n">
         <f aca="false">I41*BEN_PEDIDO-G41*(1+RECARGO)</f>
-        <v>31.0785714285714</v>
+        <v>32.1076190476191</v>
       </c>
       <c r="L41" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.111111111111111</v>
+        <v>0.121081615362892</v>
       </c>
       <c r="M41" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B41,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.0185586888406845</v>
+        <v>0.0160971476983903</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3293,31 +3329,31 @@
       </c>
       <c r="G42" s="22" t="n">
         <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>8.5</v>
+        <v>39.51</v>
       </c>
       <c r="H42" s="25" t="n">
         <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I42" s="26" t="n">
         <f aca="false">H42*RATIO</f>
-        <v>2.0952380952381</v>
+        <v>6.28571428571429</v>
       </c>
       <c r="J42" s="23" t="n">
         <f aca="false">IF(I42&gt;0,G42/I42,"")</f>
-        <v>4.05681818181818</v>
+        <v>6.28568181818182</v>
       </c>
       <c r="K42" s="23" t="n">
         <f aca="false">I42*BEN_PEDIDO-G42*(1+RECARGO)</f>
-        <v>15.0295238095238</v>
+        <v>31.0785714285714</v>
       </c>
       <c r="L42" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.182529335071708</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="M42" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B42,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.0247718383311604</v>
+        <v>0.0185586888406845</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3333,34 +3369,73 @@
       </c>
       <c r="G43" s="22" t="n">
         <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>13.63</v>
+        <v>8.5</v>
       </c>
       <c r="H43" s="25" t="n">
         <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I43" s="26" t="n">
         <f aca="false">H43*RATIO</f>
-        <v>1.04761904761905</v>
+        <v>2.0952380952381</v>
       </c>
       <c r="J43" s="23" t="n">
         <f aca="false">IF(I43&gt;0,G43/I43,"")</f>
-        <v>13.0104545454545</v>
+        <v>4.05681818181818</v>
       </c>
       <c r="K43" s="23" t="n">
         <f aca="false">I43*BEN_PEDIDO-G43*(1+RECARGO)</f>
-        <v>-1.86523809523809</v>
+        <v>15.0295238095238</v>
       </c>
       <c r="L43" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
-        <v>0.265060240963855</v>
+        <v>0.182529335071708</v>
       </c>
       <c r="M43" s="27" t="n">
         <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B43,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
+        <v>0.0247718383311604</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="25" t="n">
+        <f aca="false">COUNTIF(Creativos!$H$5:$H$16,$B44)</f>
+        <v>2</v>
+      </c>
+      <c r="G44" s="22" t="n">
+        <f aca="false">SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
+        <v>13.63</v>
+      </c>
+      <c r="H44" s="25" t="n">
+        <f aca="false">SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)</f>
+        <v>1</v>
+      </c>
+      <c r="I44" s="26" t="n">
+        <f aca="false">H44*RATIO</f>
+        <v>1.04761904761905</v>
+      </c>
+      <c r="J44" s="23" t="n">
+        <f aca="false">IF(I44&gt;0,G44/I44,"")</f>
+        <v>13.0104545454545</v>
+      </c>
+      <c r="K44" s="23" t="n">
+        <f aca="false">I44*BEN_PEDIDO-G44*(1+RECARGO)</f>
+        <v>-1.86523809523809</v>
+      </c>
+      <c r="L44" s="27" t="n">
+        <f aca="false">IFERROR(SUMIFS(Histórico!$M$5:$M$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
+        <v>0.265060240963855</v>
+      </c>
+      <c r="M44" s="27" t="n">
+        <f aca="false">IFERROR(SUMIFS(Histórico!$H$5:$H$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/SUMIFS(Histórico!$G$5:$G$5000,Histórico!$S$5:$S$5000,$B44,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA),"")</f>
         <v>0.036144578313253</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3401,8 +3476,9 @@
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="77">
+  <mergeCells count="78">
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="B5:M5"/>
@@ -3472,14 +3548,15 @@
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B36:M36"/>
-    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B37:M37"/>
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="B42:E42"/>
     <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
   </mergeCells>
   <conditionalFormatting sqref="J7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -3519,7 +3596,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K32:K34">
+  <conditionalFormatting sqref="K32:K35">
     <cfRule type="cellIs" priority="12" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>0</formula>
     </cfRule>
@@ -3527,7 +3604,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K38:K43">
+  <conditionalFormatting sqref="K39:K44">
     <cfRule type="cellIs" priority="14" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>0</formula>
     </cfRule>
@@ -3569,17 +3646,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="28" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" s="28"/>
       <c r="D4" s="28"/>
@@ -3591,19 +3668,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>31</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G5" s="18" t="s">
         <v>32</v>
@@ -3617,7 +3694,7 @@
     </row>
     <row r="6" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="29" t="str">
-        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$17,MATCH("C1",Cuerpos!$A$5:$A$17,0)),"")</f>
+        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$18,MATCH("C1",Cuerpos!$A$5:$A$18,0)),"")</f>
         <v>No la hiciste tú, pero la vas a pagar tú. Vas al taller, te piden 120 euros y te quedas dos días sin coche, por una raya que no es culpa tuya. Oye, ¿y si no hiciera falta? Me pulverizas, pasas el paño y la raya deja de verse. No lijo, relleno. Tu coche tiene el barniz que tiene. Yo no te quito ni una capa. 29 euros. Y me pagas cuando llego a tu casa. Haz clic en el enlace. Guárdame en el maletero y olvídate.</v>
       </c>
       <c r="C6" s="30" t="str">
@@ -3682,7 +3759,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">SUM(E6:E7)</f>
@@ -3703,7 +3780,7 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="35"/>
       <c r="D10" s="35"/>
@@ -3715,19 +3792,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>31</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G11" s="18" t="s">
         <v>32</v>
@@ -3741,7 +3818,7 @@
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="29" t="str">
-        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$17,MATCH("C2",Cuerpos!$A$5:$A$17,0)),"")</f>
+        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$18,MATCH("C2",Cuerpos!$A$5:$A$18,0)),"")</f>
         <v>Un dineral en el taller. La pulidora te come barniz y el del súper no hace nada. Pues no hace falta. Soy Ceralux y funciono al revés que una pulidora. Ella lija el barniz hasta igualar la raya. Yo la relleno y te dejo el barniz intacto. Pasa la uña por encima del rayón. Si se engancha, es demasiado profunda y yo no te sirvo. Si no se engancha, soy tu solución. Puesto menos de 30 euros y no pagas nada hasta tenerme en la mano. 10 minutos y ahora te quedas tranquilo de haberlo vendido por lo que vale.</v>
       </c>
       <c r="C12" s="36" t="str">
@@ -3837,7 +3914,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E15" s="33" t="n">
         <f aca="false">SUM(E12:E14)</f>
@@ -3858,7 +3935,7 @@
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="37" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" s="37"/>
       <c r="D17" s="37"/>
@@ -3870,19 +3947,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E18" s="18" t="s">
         <v>31</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G18" s="18" t="s">
         <v>32</v>
@@ -3896,7 +3973,7 @@
     </row>
     <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="29" t="str">
-        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$17,MATCH("C3",Cuerpos!$A$5:$A$17,0)),"")</f>
+        <f aca="false">IFERROR(INDEX(Cuerpos!$K$5:$K$18,MATCH("C3",Cuerpos!$A$5:$A$18,0)),"")</f>
         <v>Este es el reparador de arañazos del que habla todo el mundo. Míralo, sin cortes y sin Photoshop. Dos pulsaciones sobre el paño y lo pasamos directamente por encima del arañazo. La fórmula de nanopolímeros rellena la marca y te alisa la superficie al instante, sin lijar el barniz. Esa raya blanca, un par de pasadas y deja de verse. Funciona en cualquier color de coche, mismo resultado. No pagas nada hasta que lo tienes en la mano y lo ves funcionar. Hoy te llevas dos botes por 39,90 y el envío te sale gratis. Pagas en casa cuando te llegue. El enlace está aquí abajo.</v>
       </c>
       <c r="C19" s="38" t="str">
@@ -4116,7 +4193,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C26" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E26" s="33" t="n">
         <f aca="false">SUM(E19:E25)</f>
@@ -4274,68 +4351,68 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E4" s="39" t="s">
         <v>46</v>
       </c>
       <c r="F4" s="39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G4" s="39" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H4" s="39" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I4" s="39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L4" s="39" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M4" s="18" t="s">
         <v>31</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q4" s="18" t="s">
         <v>37</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="S4" s="18" t="s">
         <v>32</v>
@@ -4344,66 +4421,66 @@
         <v>39</v>
       </c>
       <c r="U4" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V4" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="W4" s="18" t="s">
         <v>41</v>
       </c>
       <c r="X4" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Y4" s="18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Z4" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AA4" s="18" t="s">
         <v>34</v>
       </c>
       <c r="AB4" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AC4" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>42</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G5" s="43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H5" s="43" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J5" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K5" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L5" s="44"/>
       <c r="M5" s="22" t="n">
@@ -4477,37 +4554,37 @@
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="40" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>42</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G6" s="43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H6" s="43" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J6" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K6" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L6" s="44"/>
       <c r="M6" s="22" t="n">
@@ -4581,37 +4658,37 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D7" s="49" t="s">
         <v>43</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G7" s="43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H7" s="43" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I7" s="44" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J7" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K7" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L7" s="44"/>
       <c r="M7" s="22" t="n">
@@ -4685,37 +4762,37 @@
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B8" s="36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D8" s="49" t="s">
         <v>43</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F8" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G8" s="43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H8" s="43" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" s="44" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J8" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K8" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L8" s="44"/>
       <c r="M8" s="22" t="n">
@@ -4789,37 +4866,37 @@
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="48" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B9" s="36" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D9" s="49" t="s">
         <v>43</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F9" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G9" s="43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H9" s="43" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I9" s="44" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J9" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K9" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L9" s="44"/>
       <c r="M9" s="22" t="n">
@@ -4893,35 +4970,35 @@
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="50" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G10" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H10" s="43" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I10" s="44"/>
       <c r="J10" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K10" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L10" s="44"/>
       <c r="M10" s="22" t="n">
@@ -4995,35 +5072,35 @@
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="50" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D11" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G11" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H11" s="43" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K11" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L11" s="44"/>
       <c r="M11" s="22" t="n">
@@ -5097,35 +5174,35 @@
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="50" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D12" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F12" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G12" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H12" s="43" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I12" s="44"/>
       <c r="J12" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K12" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L12" s="44"/>
       <c r="M12" s="22" t="n">
@@ -5199,35 +5276,35 @@
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="50" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D13" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F13" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G13" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H13" s="43" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K13" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L13" s="44"/>
       <c r="M13" s="22" t="n">
@@ -5301,35 +5378,35 @@
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="50" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D14" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F14" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G14" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H14" s="43" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I14" s="44"/>
       <c r="J14" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K14" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L14" s="44"/>
       <c r="M14" s="22" t="n">
@@ -5403,35 +5480,35 @@
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="50" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D15" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E15" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F15" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G15" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H15" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I15" s="44"/>
       <c r="J15" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K15" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L15" s="44"/>
       <c r="M15" s="22" t="n">
@@ -5505,35 +5582,35 @@
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="50" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D16" s="51" t="s">
         <v>44</v>
       </c>
       <c r="E16" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F16" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G16" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H16" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I16" s="44"/>
       <c r="J16" s="45" t="n">
         <v>46300</v>
       </c>
       <c r="K16" s="46" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L16" s="44"/>
       <c r="M16" s="22" t="n">
@@ -5670,7 +5747,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E36" type="list">
-      <formula1>Cuerpos!$A$5:$A$17</formula1>
+      <formula1>Cuerpos!$A$5:$A$18</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G36" type="list">
@@ -5694,7 +5771,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -5719,59 +5796,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="39" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E4" s="39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F4" s="39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G4" s="39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H4" s="39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I4" s="39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J4" s="39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="N4" s="39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O4" s="39" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P4" s="18" t="s">
         <v>36</v>
@@ -5791,32 +5868,32 @@
     </row>
     <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C5" s="44" t="s">
         <v>42</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G5" s="44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H5" s="44"/>
       <c r="I5" s="44" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K5" s="52" t="str">
         <f aca="false">TRIM(E5&amp;" "&amp;F5&amp;" "&amp;G5&amp;" "&amp;H5&amp;" "&amp;I5&amp;" "&amp;J5)</f>
@@ -5831,7 +5908,7 @@
         <v>33</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="O5" s="44"/>
       <c r="P5" s="25" t="n">
@@ -5857,34 +5934,34 @@
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C6" s="44" t="s">
         <v>43</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G6" s="44" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H6" s="44" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K6" s="52" t="str">
         <f aca="false">TRIM(E6&amp;" "&amp;F6&amp;" "&amp;G6&amp;" "&amp;H6&amp;" "&amp;I6&amp;" "&amp;J6)</f>
@@ -5899,10 +5976,10 @@
         <v>38</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="O6" s="44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="P6" s="25" t="n">
         <f aca="false">IF(A6="","",COUNTIF(Creativos!$E$5:$E$16,A6))</f>
@@ -5927,34 +6004,34 @@
     </row>
     <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C7" s="44" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G7" s="44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H7" s="44" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I7" s="44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J7" s="44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K7" s="52" t="str">
         <f aca="false">TRIM(E7&amp;" "&amp;F7&amp;" "&amp;G7&amp;" "&amp;H7&amp;" "&amp;I7&amp;" "&amp;J7)</f>
@@ -5969,10 +6046,10 @@
         <v>41</v>
       </c>
       <c r="N7" s="44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O7" s="44" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P7" s="25" t="n">
         <f aca="false">IF(A7="","",COUNTIF(Creativos!$E$5:$E$16,A7))</f>
@@ -5995,50 +6072,74 @@
         <v>76.3504761904762</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="43"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="44"/>
-      <c r="J8" s="44"/>
+    <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="43" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="F8" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="H8" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="I8" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="J8" s="44" t="s">
+        <v>178</v>
+      </c>
       <c r="K8" s="52" t="str">
         <f aca="false">TRIM(E8&amp;" "&amp;F8&amp;" "&amp;G8&amp;" "&amp;H8&amp;" "&amp;I8&amp;" "&amp;J8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="25" t="str">
+        <v>Y eso sin quedarte tirado dos días sin coche. Y sí, ya lo has probado: la pasta de dientes, lo del súper, los rotuladores esos que anuncian... y la raya ahí sigue. Dos pulsaciones sobre el paño, y lo pasamos directamente por encima del arañazo. La fórmula de nanopolímeros rellena la marca y te alisa la superficie al instante, sin estropear el barniz. ¿Esa raya blanca que ves cada vez que te acercas al coche? Un par de pasadas, y deja de verse. Te preguntarás si te va a servir a ti. Pasa la uña por la raya. Si no se engancha, esto es para ti. Si se engancha, es de taller. Así de claro. Por su lanzamiento, solo hasta el 31 de octubre, te llevas dos botes por 39,90. El segundo te sale a menos de diez euros. Envío gratis, y no pagas nada hasta que te llega a casa. Pulsa el enlace de abajo y pídelo ahora.</v>
+      </c>
+      <c r="L8" s="25" t="n">
         <f aca="false">IF(K8="","",LEN(K8)-LEN(SUBSTITUTE(K8," ",""))+1)</f>
-        <v/>
-      </c>
-      <c r="M8" s="25" t="str">
+        <v>159</v>
+      </c>
+      <c r="M8" s="25" t="n">
         <f aca="false">IF(L8="","",ROUND(L8/2.6,0))</f>
-        <v/>
-      </c>
-      <c r="N8" s="44"/>
-      <c r="O8" s="44"/>
-      <c r="P8" s="25" t="str">
+        <v>61</v>
+      </c>
+      <c r="N8" s="44" t="s">
+        <v>167</v>
+      </c>
+      <c r="O8" s="44" t="s">
+        <v>179</v>
+      </c>
+      <c r="P8" s="25" t="n">
         <f aca="false">IF(A8="","",COUNTIF(Creativos!$E$5:$E$16,A8))</f>
-        <v/>
-      </c>
-      <c r="Q8" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="22" t="n">
         <f aca="false">IF(A8="","",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$R$5:$R$5000,$A8,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA))</f>
-        <v/>
-      </c>
-      <c r="R8" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="R8" s="25" t="n">
         <f aca="false">IF(A8="","",SUMIFS(Histórico!$L$5:$L$5000,Histórico!$R$5:$R$5000,$A8,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S8" s="23" t="str">
         <f aca="false">IF(N(R8)*RATIO&gt;0,Q8/(R8*RATIO),"")</f>
         <v/>
       </c>
-      <c r="T8" s="23" t="str">
+      <c r="T8" s="23" t="n">
         <f aca="false">IF(A8="","",R8*RATIO*BEN_PEDIDO-Q8*(1+RECARGO))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6455,8 +6556,54 @@
         <v/>
       </c>
     </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="43"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="52" t="str">
+        <f aca="false">TRIM(E18&amp;" "&amp;F18&amp;" "&amp;G18&amp;" "&amp;H18&amp;" "&amp;I18&amp;" "&amp;J18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="25" t="str">
+        <f aca="false">IF(K18="","",LEN(K18)-LEN(SUBSTITUTE(K18," ",""))+1)</f>
+        <v/>
+      </c>
+      <c r="M18" s="25" t="str">
+        <f aca="false">IF(L18="","",ROUND(L18/2.6,0))</f>
+        <v/>
+      </c>
+      <c r="N18" s="44"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="25" t="str">
+        <f aca="false">IF(A18="","",COUNTIF(Creativos!$E$5:$E$16,A18))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="22" t="str">
+        <f aca="false">IF(A18="","",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$R$5:$R$5000,$A18,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA))</f>
+        <v/>
+      </c>
+      <c r="R18" s="25" t="str">
+        <f aca="false">IF(A18="","",SUMIFS(Histórico!$L$5:$L$5000,Histórico!$R$5:$R$5000,$A18,Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA))</f>
+        <v/>
+      </c>
+      <c r="S18" s="23" t="str">
+        <f aca="false">IF(N(R18)*RATIO&gt;0,Q18/(R18*RATIO),"")</f>
+        <v/>
+      </c>
+      <c r="T18" s="23" t="str">
+        <f aca="false">IF(A18="","",R18*RATIO*BEN_PEDIDO-Q18*(1+RECARGO))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="T5:T17">
+  <conditionalFormatting sqref="T5:T18">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>0</formula>
     </cfRule>
@@ -6479,27 +6626,27 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:E12"/>
+  <dimension ref="B1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>47</v>
@@ -6510,10 +6657,13 @@
       <c r="E4" s="18" t="s">
         <v>49</v>
       </c>
+      <c r="F4" s="18" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="53" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C5" s="54" t="n">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6527,10 +6677,14 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>—</v>
       </c>
+      <c r="F5" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B5,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="53" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" s="54" t="str">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6544,10 +6698,14 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>—</v>
       </c>
+      <c r="F6" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B6,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="53" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7" s="54" t="str">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6561,10 +6719,14 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>8.16518181818182</v>
       </c>
+      <c r="F7" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B7,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="53" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="54" t="str">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6578,10 +6740,14 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>6.28568181818182</v>
       </c>
+      <c r="F8" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B8,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="53" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C9" s="54" t="str">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6595,10 +6761,14 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>4.05681818181818</v>
       </c>
+      <c r="F9" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B9,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="53" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="54" t="str">
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C1",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
@@ -6612,14 +6782,18 @@
         <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C3",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
         <v>13.0104545454545</v>
       </c>
+      <c r="F10" s="54" t="str">
+        <f aca="false">IF(SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"—",IF(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)=0,"sin ventas",SUMIFS(Histórico!$F$5:$F$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)/(SUMIFS(Histórico!$L$5:$L$5000,Histórico!$S$5:$S$5000,$B10,Histórico!$R$5:$R$5000,"C4",Histórico!$A$5:$A$5000,"&gt;="&amp;DESDE,Histórico!$A$5:$A$5000,"&lt;="&amp;HASTA)*RATIO)))</f>
+        <v>—</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:E10">
+  <conditionalFormatting sqref="C5:F10">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>AND(ISNUMBER(C5),C5&lt;=UMB_ESC*CPA_BE)</formula>
     </cfRule>
@@ -6663,74 +6837,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>28</v>
       </c>
       <c r="D4" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="18" t="s">
         <v>72</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>31</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="R4" s="18" t="s">
         <v>46</v>
       </c>
       <c r="S4" s="18" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="T4" s="18" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="U4" s="18" t="s">
         <v>41</v>
@@ -6739,7 +6913,7 @@
         <v>40</v>
       </c>
       <c r="W4" s="18" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6747,16 +6921,16 @@
         <v>46300</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E5" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F5" s="22" t="n">
         <v>15.67</v>
@@ -6824,16 +6998,16 @@
         <v>46300</v>
       </c>
       <c r="B6" s="55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C6" s="56" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D6" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F6" s="22" t="n">
         <v>27.53</v>
@@ -6901,16 +7075,16 @@
         <v>46300</v>
       </c>
       <c r="B7" s="55" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D7" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E7" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F7" s="22" t="n">
         <v>1.28</v>
@@ -6978,16 +7152,16 @@
         <v>46300</v>
       </c>
       <c r="B8" s="55" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C8" s="56" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D8" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F8" s="22" t="n">
         <v>7.7</v>
@@ -7055,16 +7229,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="55" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C9" s="56" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D9" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F9" s="22" t="n">
         <v>0.04</v>
@@ -7132,16 +7306,16 @@
         <v>46300</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D10" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E10" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F10" s="22" t="n">
         <v>0.72</v>
@@ -7209,16 +7383,16 @@
         <v>46300</v>
       </c>
       <c r="B11" s="55" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C11" s="56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D11" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E11" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F11" s="22" t="n">
         <v>5.07</v>
@@ -7286,16 +7460,16 @@
         <v>46300</v>
       </c>
       <c r="B12" s="55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" s="56" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D12" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F12" s="22" t="n">
         <v>3.39</v>
@@ -7363,16 +7537,16 @@
         <v>46300</v>
       </c>
       <c r="B13" s="55" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D13" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F13" s="22" t="n">
         <v>1.35</v>
@@ -7440,16 +7614,16 @@
         <v>46300</v>
       </c>
       <c r="B14" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E14" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F14" s="22" t="n">
         <v>4.09</v>
@@ -7517,16 +7691,16 @@
         <v>46300</v>
       </c>
       <c r="B15" s="55" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D15" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E15" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F15" s="22" t="n">
         <v>0.09</v>
@@ -7594,16 +7768,16 @@
         <v>46300</v>
       </c>
       <c r="B16" s="55" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E16" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F16" s="22" t="n">
         <v>0.74</v>
@@ -7671,16 +7845,16 @@
         <v>46301</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" s="56" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D17" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E17" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F17" s="22" t="n">
         <v>48.97</v>
@@ -7748,16 +7922,16 @@
         <v>46301</v>
       </c>
       <c r="B18" s="55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D18" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E18" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F18" s="22" t="n">
         <v>4.97</v>
@@ -7825,16 +7999,16 @@
         <v>46301</v>
       </c>
       <c r="B19" s="55" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C19" s="56" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D19" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E19" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F19" s="22" t="n">
         <v>0.47</v>
@@ -7902,16 +8076,16 @@
         <v>46301</v>
       </c>
       <c r="B20" s="55" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C20" s="56" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D20" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E20" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F20" s="22" t="n">
         <v>0.38</v>
@@ -7979,16 +8153,16 @@
         <v>46301</v>
       </c>
       <c r="B21" s="55" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C21" s="56" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D21" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E21" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F21" s="22" t="n">
         <v>0.01</v>
@@ -8056,16 +8230,16 @@
         <v>46301</v>
       </c>
       <c r="B22" s="55" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C22" s="56" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D22" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E22" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F22" s="22" t="n">
         <v>0.01</v>
@@ -8133,16 +8307,16 @@
         <v>46301</v>
       </c>
       <c r="B23" s="55" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F23" s="22" t="n">
         <v>5.13</v>
@@ -8210,16 +8384,16 @@
         <v>46301</v>
       </c>
       <c r="B24" s="55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D24" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E24" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F24" s="22" t="n">
         <v>3.48</v>
@@ -8287,16 +8461,16 @@
         <v>46301</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C25" s="56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D25" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E25" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F25" s="22" t="n">
         <v>1.25</v>
@@ -8364,16 +8538,16 @@
         <v>46301</v>
       </c>
       <c r="B26" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D26" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F26" s="22" t="n">
         <v>2.45</v>
@@ -8441,16 +8615,16 @@
         <v>46301</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C27" s="56" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D27" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E27" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F27" s="22" t="n">
         <v>1.51</v>
@@ -8518,16 +8692,16 @@
         <v>46301</v>
       </c>
       <c r="B28" s="55" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D28" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E28" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F28" s="22" t="n">
         <v>1.55</v>
@@ -8595,16 +8769,16 @@
         <v>46302</v>
       </c>
       <c r="B29" s="55" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D29" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E29" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F29" s="22" t="n">
         <v>20.9</v>
@@ -8672,16 +8846,16 @@
         <v>46302</v>
       </c>
       <c r="B30" s="55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D30" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E30" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F30" s="22" t="n">
         <v>5.2</v>
@@ -8749,16 +8923,16 @@
         <v>46302</v>
       </c>
       <c r="B31" s="55" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="56" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D31" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E31" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F31" s="22" t="n">
         <v>0.06</v>
@@ -8826,16 +9000,16 @@
         <v>46302</v>
       </c>
       <c r="B32" s="55" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D32" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E32" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F32" s="22" t="n">
         <v>0.37</v>
@@ -8903,16 +9077,16 @@
         <v>46302</v>
       </c>
       <c r="B33" s="55" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33" s="56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D33" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E33" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F33" s="22" t="n">
         <v>2.7</v>
@@ -8980,16 +9154,16 @@
         <v>46302</v>
       </c>
       <c r="B34" s="55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D34" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E34" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F34" s="22" t="n">
         <v>3.43</v>
@@ -9057,16 +9231,16 @@
         <v>46302</v>
       </c>
       <c r="B35" s="55" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D35" s="46" t="s">
         <v>42</v>
       </c>
       <c r="E35" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F35" s="22" t="n">
         <v>0.77</v>
@@ -9134,16 +9308,16 @@
         <v>46302</v>
       </c>
       <c r="B36" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C36" s="56" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D36" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E36" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F36" s="22" t="n">
         <v>2.63</v>
@@ -9211,16 +9385,16 @@
         <v>46302</v>
       </c>
       <c r="B37" s="55" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C37" s="56" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D37" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E37" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F37" s="22" t="n">
         <v>0.75</v>
@@ -9288,16 +9462,16 @@
         <v>46302</v>
       </c>
       <c r="B38" s="55" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D38" s="46" t="s">
         <v>43</v>
       </c>
       <c r="E38" s="57" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F38" s="22" t="n">
         <v>0.55</v>
@@ -9388,26 +9562,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>31</v>
@@ -9517,159 +9691,159 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="18" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="D3" s="18"/>
       <c r="E3" s="18" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="62" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="C4" s="63" t="n">
         <v>11.23</v>
       </c>
       <c r="E4" s="64" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="F4" s="65" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="62" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="C5" s="63" t="n">
         <v>11.23</v>
       </c>
       <c r="E5" s="64" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="F5" s="65" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="62" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C6" s="66" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="64" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="F6" s="65" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="62" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46300</v>
       </c>
       <c r="E7" s="64" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="F7" s="65" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="62" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C8" s="66" t="n">
         <v>0.75</v>
       </c>
       <c r="E8" s="64" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="F8" s="65" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="62" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C9" s="67" t="n">
         <v>1.5</v>
       </c>
       <c r="E9" s="64" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="F9" s="65" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="62" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C10" s="67" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="64" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="F10" s="65" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="62" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="C11" s="61" t="n">
         <v>800</v>
       </c>
       <c r="E11" s="64" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="F11" s="65" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="68" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="69" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="62" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C16" s="62" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -9697,102 +9871,102 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="70" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="71" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="71" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="71" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="71" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="71" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="71" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="70" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="71" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="71" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="70" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="71" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="71" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="71" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="71" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="70" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="71" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="71" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="71" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>